<commit_message>
WIP: livrables de la flotte (données, gouvernance, DA, site, contenus, légal, ops, pilotage, agents)
Snapshot intermédiaire pendant le build ; intégrations et orchestration encore en cours.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MykNGMmExNHnMWtHwWJ6jS
</commit_message>
<xml_diff>
--- a/docs/03-finance/tresorerie_13_semaines.xlsx
+++ b/docs/03-finance/tresorerie_13_semaines.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="103">
   <si>
     <t xml:space="preserve">Trésorerie glissante 13 semaines — mode d'emploi</t>
   </si>
@@ -57,19 +57,25 @@
     <t xml:space="preserve">5.</t>
   </si>
   <si>
-    <t xml:space="preserve">Alerte (ligne 49) : SOLDE NÉGATIF, SOUS RÉSERVE MINI (solde &lt; B7), PRÉCOMMANDES NON COUVERTES (solde − réserve précommandes − réserve mini &lt; 0). Toute alerte bloque les achats « prévus » jusqu'à arbitrage.</t>
+    <t xml:space="preserve">Alerte de clôture (ligne 49) : SOLDE NÉGATIF, SOUS RÉSERVE MINI (solde &lt; B7), PRÉCOMMANDES NON COUVERTES (solde − réserve précommandes − réserve mini &lt; 0).</t>
   </si>
   <si>
     <t xml:space="preserve">6.</t>
   </si>
   <si>
-    <t xml:space="preserve">La feuille « Exemple FICTIF » illustre le plan 90 jours du BP §9 avec des montants inventés : ne jamais l'utiliser comme prévision.</t>
+    <t xml:space="preserve">STOP-LOSS CASH (lignes 50-51) : la réserve minimale B7 vaut 1 600 CHF, la réserve de trésorerie du budget BP §3. Une semaine qui s'ouvre après une clôture en alerte est en stop-loss : plus aucun achat prévu ni aucune publicité (ligne 51 = montants à supprimer ou décaler). Les achats engagés restent dus. Seule la propriétaire peut modifier B7.</t>
   </si>
   <si>
     <t xml:space="preserve">7.</t>
   </si>
   <si>
-    <t xml:space="preserve">Le moteur Python pokeshop.treasury (plan_from_weekly_inputs + build_forecast) reproduit exactement ces calculs pour le tableau de bord et les tests.</t>
+    <t xml:space="preserve">La feuille « Exemple FICTIF » applique le budget BP §3 et le plan 90 jours BP §9 avec des montants inventés : ne jamais l'utiliser comme prévision. Elle montre la réserve entamée dès la semaine 5 (charges fixes non budgétées).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le moteur Python pokeshop.treasury (plan_from_weekly_inputs + build_forecast) reproduit exactement ces calculs pour le tableau de bord et les tests ; enforce_cash_stoploss=True y simule en plus l'application du blocage.</t>
   </si>
   <si>
     <t xml:space="preserve">Légende</t>
@@ -81,7 +87,7 @@
     <t xml:space="preserve">Formule (texte noir) — ne pas écraser</t>
   </si>
   <si>
-    <t xml:space="preserve">Alerte de trésorerie</t>
+    <t xml:space="preserve">Alerte de trésorerie ou stop-loss cash</t>
   </si>
   <si>
     <t xml:space="preserve">Validation humaine requise</t>
@@ -90,7 +96,10 @@
     <t xml:space="preserve">☐</t>
   </si>
   <si>
-    <t xml:space="preserve">Montant de la réserve minimale (B7) et règle d'arbitrage en cas d'alerte.</t>
+    <t xml:space="preserve">Seuil du stop-loss cash (B7, 1 600 CHF par défaut) : toute modification est une décision de la propriétaire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financement des charges fixes d'avant l'ouverture (≈ 400 à 600 CHF), absentes du budget de 8 000 CHF.</t>
   </si>
   <si>
     <t xml:space="preserve">Délai réel de versement et frais du PSP (contrat, paiements tests carte et TWINT).</t>
@@ -126,10 +135,10 @@
     <t xml:space="preserve">Relevé bancaire du jour</t>
   </si>
   <si>
-    <t xml:space="preserve">Réserve minimale (CHF)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plancher à ne pas franchir — décision de la responsable</t>
+    <t xml:space="preserve">Réserve minimale = seuil du stop-loss cash (CHF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BP §3 : réserve 1 600 CHF. Sous ce seuil (solde − précommandes) : plus d'achat prévu ni de pub</t>
   </si>
   <si>
     <t xml:space="preserve">Frais PSP proportionnels</t>
@@ -258,7 +267,7 @@
     <t xml:space="preserve">Solde de clôture</t>
   </si>
   <si>
-    <t xml:space="preserve">RÉSERVES ET ALERTE</t>
+    <t xml:space="preserve">RÉSERVES, ALERTE ET STOP-LOSS CASH</t>
   </si>
   <si>
     <t xml:space="preserve">Précommandes livrées (réserve libérée, TTC)</t>
@@ -267,13 +276,19 @@
     <t xml:space="preserve">Réserve précommandes (fin de semaine)</t>
   </si>
   <si>
-    <t xml:space="preserve">Réserve minimale</t>
+    <t xml:space="preserve">Réserve minimale = seuil du stop-loss cash</t>
   </si>
   <si>
     <t xml:space="preserve">Disponible pour de nouveaux achats</t>
   </si>
   <si>
-    <t xml:space="preserve">Alerte</t>
+    <t xml:space="preserve">Alerte (clôture)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stop-loss cash actif en début de semaine ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Achats prévus + publicité à bloquer (mandat)</t>
   </si>
   <si>
     <t xml:space="preserve">SYNTHÈSE</t>
@@ -285,7 +300,7 @@
     <t xml:space="preserve">Semaine du solde le plus bas</t>
   </si>
   <si>
-    <t xml:space="preserve">Nombre de semaines en alerte</t>
+    <t xml:space="preserve">Nombre de semaines en alerte (clôture)</t>
   </si>
   <si>
     <t xml:space="preserve">Versements PSP en transit à la fin de l'horizon</t>
@@ -298,6 +313,18 @@
   </si>
   <si>
     <t xml:space="preserve">Hors impôt préalable déductible : le décompte réel est établi avec la fiduciaire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semaines ouvertes en stop-loss cash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Première semaine en stop-loss cash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Achats prévus + publicité à bloquer (13 semaines)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montants à supprimer ou à décaler : le mandat interdit tout achat prévu et toute publicité tant que le stop-loss cash est actif. Les achats déjà engagés restent dus.</t>
   </si>
   <si>
     <t xml:space="preserve">Trésorerie 13 semaines — {{NOM_BOUTIQUE}}</t>
@@ -872,7 +899,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -945,66 +972,82 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+    <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>16</v>
       </c>
+      <c r="B11" s="4" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6"/>
-      <c r="B13" s="7" t="s">
-        <v>17</v>
+      <c r="A13" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="6"/>
+      <c r="B14" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="n">
         <v>1234.5</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
       <c r="B15" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
         <v>20</v>
       </c>
     </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9"/>
+      <c r="B16" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1023,7 +1066,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:P57"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -1034,17 +1077,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
@@ -1064,7 +1107,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -1084,95 +1127,95 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>46300</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B6" s="16" t="n">
         <v>8000</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B7" s="16" t="n">
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>0.025</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>0.3</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B11" s="19" t="n">
         <v>0.081</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B12" s="16" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -1192,7 +1235,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B14" s="20"/>
       <c r="C14" s="20" t="n">
@@ -1235,12 +1278,12 @@
         <v>13</v>
       </c>
       <c r="P14" s="20" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C15" s="21" t="n">
         <f aca="false">IF($B$5="","",$B$5+7*(C$14-1))</f>
@@ -1297,7 +1340,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C16" s="21" t="n">
         <f aca="false">IF($B$5="","",C15+6)</f>
@@ -1354,7 +1397,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
@@ -1392,7 +1435,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="18"/>
@@ -1430,7 +1473,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
@@ -1441,22 +1484,20 @@
       <c r="I19" s="16"/>
       <c r="J19" s="16"/>
       <c r="K19" s="16" t="n">
-        <v>479.4</v>
-      </c>
-      <c r="L19" s="16" t="n">
-        <v>319.6</v>
-      </c>
+        <v>639.2</v>
+      </c>
+      <c r="L19" s="16"/>
       <c r="M19" s="16"/>
       <c r="N19" s="16"/>
       <c r="O19" s="16"/>
       <c r="P19" s="22" t="n">
         <f aca="false">SUM(C19:O19)</f>
-        <v>799</v>
+        <v>639.2</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="18"/>
@@ -1467,22 +1508,20 @@
       <c r="I20" s="18"/>
       <c r="J20" s="18"/>
       <c r="K20" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="L20" s="18" t="n">
-        <v>4</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="L20" s="18"/>
       <c r="M20" s="18"/>
       <c r="N20" s="18"/>
       <c r="O20" s="18"/>
       <c r="P20" s="23" t="n">
         <f aca="false">SUM(C20:O20)</f>
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C21" s="24" t="n">
         <f aca="false">(C17+C19)*$B$8+(C18+C20)*$B$9</f>
@@ -1518,11 +1557,11 @@
       </c>
       <c r="K21" s="24" t="n">
         <f aca="false">(K17+K19)*$B$8+(K18+K20)*$B$9</f>
-        <v>35.465</v>
+        <v>40.06</v>
       </c>
       <c r="L21" s="24" t="n">
         <f aca="false">(L17+L19)*$B$8+(L18+L20)*$B$9</f>
-        <v>32.955</v>
+        <v>23.765</v>
       </c>
       <c r="M21" s="24" t="n">
         <f aca="false">(M17+M19)*$B$8+(M18+M20)*$B$9</f>
@@ -1538,12 +1577,12 @@
       </c>
       <c r="P21" s="22" t="n">
         <f aca="false">SUM(C21:O21)</f>
-        <v>191.65</v>
+        <v>187.055</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C22" s="24" t="n">
         <f aca="false">C17+C19-C21</f>
@@ -1579,11 +1618,11 @@
       </c>
       <c r="K22" s="24" t="n">
         <f aca="false">K17+K19-K21</f>
-        <v>1215.135</v>
+        <v>1370.34</v>
       </c>
       <c r="L22" s="24" t="n">
         <f aca="false">L17+L19-L21</f>
-        <v>1129.245</v>
+        <v>818.835</v>
       </c>
       <c r="M22" s="24" t="n">
         <f aca="false">M17+M19-M21</f>
@@ -1599,12 +1638,12 @@
       </c>
       <c r="P22" s="22" t="n">
         <f aca="false">SUM(C22:O22)</f>
-        <v>6598.35</v>
+        <v>6443.145</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
@@ -1624,7 +1663,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C24" s="24" t="n">
         <f aca="false">IF(C$14-$B$10&gt;=1,INDEX($C$22:$O$22,C$14-$B$10),0)</f>
@@ -1664,11 +1703,11 @@
       </c>
       <c r="L24" s="24" t="n">
         <f aca="false">IF(L$14-$B$10&gt;=1,INDEX($C$22:$O$22,L$14-$B$10),0)</f>
-        <v>1215.135</v>
+        <v>1370.34</v>
       </c>
       <c r="M24" s="24" t="n">
         <f aca="false">IF(M$14-$B$10&gt;=1,INDEX($C$22:$O$22,M$14-$B$10),0)</f>
-        <v>1129.245</v>
+        <v>818.835</v>
       </c>
       <c r="N24" s="24" t="n">
         <f aca="false">IF(N$14-$B$10&gt;=1,INDEX($C$22:$O$22,N$14-$B$10),0)</f>
@@ -1680,12 +1719,12 @@
       </c>
       <c r="P24" s="22" t="n">
         <f aca="false">SUM(C24:O24)</f>
-        <v>5481.1875</v>
+        <v>5325.9825</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
@@ -1707,7 +1746,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
@@ -1729,7 +1768,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="25" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C27" s="22" t="n">
         <f aca="false">C24+C25+C26</f>
@@ -1769,11 +1808,11 @@
       </c>
       <c r="L27" s="22" t="n">
         <f aca="false">L24+L25+L26</f>
-        <v>1215.135</v>
+        <v>1370.34</v>
       </c>
       <c r="M27" s="22" t="n">
         <f aca="false">M24+M25+M26</f>
-        <v>1129.245</v>
+        <v>818.835</v>
       </c>
       <c r="N27" s="22" t="n">
         <f aca="false">N24+N25+N26</f>
@@ -1785,12 +1824,12 @@
       </c>
       <c r="P27" s="22" t="n">
         <f aca="false">SUM(C27:O27)</f>
-        <v>5481.1875</v>
+        <v>5325.9825</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
@@ -1810,7 +1849,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
@@ -1821,24 +1860,22 @@
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
       <c r="I29" s="16"/>
-      <c r="J29" s="16" t="n">
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="16" t="n">
         <v>900</v>
       </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16" t="n">
-        <v>650</v>
-      </c>
-      <c r="M29" s="16"/>
       <c r="N29" s="16"/>
       <c r="O29" s="16"/>
       <c r="P29" s="22" t="n">
         <f aca="false">SUM(C29:O29)</f>
-        <v>4550</v>
+        <v>3900</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
@@ -1850,19 +1887,19 @@
       <c r="J30" s="16"/>
       <c r="K30" s="16"/>
       <c r="L30" s="16"/>
-      <c r="M30" s="16" t="n">
-        <v>1200</v>
-      </c>
-      <c r="N30" s="16"/>
+      <c r="M30" s="16"/>
+      <c r="N30" s="16" t="n">
+        <v>650</v>
+      </c>
       <c r="O30" s="16"/>
       <c r="P30" s="22" t="n">
         <f aca="false">SUM(C30:O30)</f>
-        <v>1200</v>
+        <v>650</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
@@ -1886,7 +1923,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
@@ -1924,7 +1961,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C33" s="16"/>
       <c r="D33" s="16"/>
@@ -1948,7 +1985,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C34" s="16"/>
       <c r="D34" s="16"/>
@@ -1972,7 +2009,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
@@ -1983,15 +2020,15 @@
       <c r="I35" s="16" t="n">
         <v>150</v>
       </c>
-      <c r="J35" s="16" t="n">
+      <c r="J35" s="16"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16" t="n">
+        <v>150</v>
+      </c>
+      <c r="M35" s="16"/>
+      <c r="N35" s="16" t="n">
         <v>200</v>
       </c>
-      <c r="K35" s="16" t="n">
-        <v>150</v>
-      </c>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="16"/>
       <c r="O35" s="16"/>
       <c r="P35" s="22" t="n">
         <f aca="false">SUM(C35:O35)</f>
@@ -2000,7 +2037,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C36" s="16" t="n">
         <v>400</v>
@@ -2014,23 +2051,21 @@
       <c r="H36" s="16"/>
       <c r="I36" s="16"/>
       <c r="J36" s="16"/>
-      <c r="K36" s="16" t="n">
+      <c r="K36" s="16"/>
+      <c r="L36" s="16" t="n">
         <v>400</v>
       </c>
-      <c r="L36" s="16"/>
       <c r="M36" s="16"/>
       <c r="N36" s="16"/>
-      <c r="O36" s="16" t="n">
-        <v>400</v>
-      </c>
+      <c r="O36" s="16"/>
       <c r="P36" s="22" t="n">
         <f aca="false">SUM(C36:O36)</f>
-        <v>1600</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C37" s="16" t="n">
         <v>1100</v>
@@ -2058,7 +2093,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>
@@ -2080,7 +2115,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="25" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C39" s="22" t="n">
         <f aca="false">SUM(C29:C38)</f>
@@ -2112,36 +2147,36 @@
       </c>
       <c r="J39" s="22" t="n">
         <f aca="false">SUM(J29:J38)</f>
-        <v>1154</v>
+        <v>54</v>
       </c>
       <c r="K39" s="22" t="n">
         <f aca="false">SUM(K29:K38)</f>
-        <v>716.9</v>
+        <v>166.9</v>
       </c>
       <c r="L39" s="22" t="n">
         <f aca="false">SUM(L29:L38)</f>
-        <v>731</v>
+        <v>631</v>
       </c>
       <c r="M39" s="22" t="n">
         <f aca="false">SUM(M29:M38)</f>
-        <v>1369.9</v>
+        <v>1069.9</v>
       </c>
       <c r="N39" s="22" t="n">
         <f aca="false">SUM(N29:N38)</f>
-        <v>90</v>
+        <v>940</v>
       </c>
       <c r="O39" s="22" t="n">
         <f aca="false">SUM(O29:O38)</f>
-        <v>658</v>
+        <v>258</v>
       </c>
       <c r="P39" s="22" t="n">
         <f aca="false">SUM(C39:O39)</f>
-        <v>11641.8</v>
+        <v>10041.8</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
@@ -2161,7 +2196,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C41" s="24" t="n">
         <f aca="false">$B$6</f>
@@ -2197,23 +2232,23 @@
       </c>
       <c r="K41" s="24" t="n">
         <f aca="false">J43</f>
-        <v>668.645</v>
+        <v>1768.645</v>
       </c>
       <c r="L41" s="24" t="n">
         <f aca="false">K43</f>
-        <v>497.31</v>
+        <v>2147.31</v>
       </c>
       <c r="M41" s="24" t="n">
         <f aca="false">L43</f>
-        <v>981.445</v>
+        <v>2886.65</v>
       </c>
       <c r="N41" s="24" t="n">
         <f aca="false">M43</f>
-        <v>740.79</v>
+        <v>2635.585</v>
       </c>
       <c r="O41" s="24" t="n">
         <f aca="false">N43</f>
-        <v>1591.8825</v>
+        <v>2636.6775</v>
       </c>
       <c r="P41" s="22" t="n">
         <f aca="false">C41</f>
@@ -2222,7 +2257,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C42" s="26" t="n">
         <f aca="false">C27-C39</f>
@@ -2254,36 +2289,36 @@
       </c>
       <c r="J42" s="26" t="n">
         <f aca="false">J27-J39</f>
-        <v>-681.1625</v>
+        <v>418.8375</v>
       </c>
       <c r="K42" s="26" t="n">
         <f aca="false">K27-K39</f>
-        <v>-171.335</v>
+        <v>378.665</v>
       </c>
       <c r="L42" s="26" t="n">
         <f aca="false">L27-L39</f>
-        <v>484.135</v>
+        <v>739.34</v>
       </c>
       <c r="M42" s="26" t="n">
         <f aca="false">M27-M39</f>
-        <v>-240.655</v>
+        <v>-251.065</v>
       </c>
       <c r="N42" s="26" t="n">
         <f aca="false">N27-N39</f>
-        <v>851.0925</v>
+        <v>1.09249999999997</v>
       </c>
       <c r="O42" s="26" t="n">
         <f aca="false">O27-O39</f>
-        <v>247.505</v>
+        <v>647.505</v>
       </c>
       <c r="P42" s="22" t="n">
         <f aca="false">SUM(C42:O42)</f>
-        <v>-6160.6125</v>
+        <v>-4715.8175</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="25" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C43" s="27" t="n">
         <f aca="false">C41+C42</f>
@@ -2315,36 +2350,36 @@
       </c>
       <c r="J43" s="27" t="n">
         <f aca="false">J41+J42</f>
-        <v>668.645</v>
+        <v>1768.645</v>
       </c>
       <c r="K43" s="27" t="n">
         <f aca="false">K41+K42</f>
-        <v>497.31</v>
+        <v>2147.31</v>
       </c>
       <c r="L43" s="27" t="n">
         <f aca="false">L41+L42</f>
-        <v>981.445</v>
+        <v>2886.65</v>
       </c>
       <c r="M43" s="27" t="n">
         <f aca="false">M41+M42</f>
-        <v>740.79</v>
+        <v>2635.585</v>
       </c>
       <c r="N43" s="27" t="n">
         <f aca="false">N41+N42</f>
-        <v>1591.8825</v>
+        <v>2636.6775</v>
       </c>
       <c r="O43" s="27" t="n">
         <f aca="false">O41+O42</f>
-        <v>1839.3875</v>
+        <v>3284.1825</v>
       </c>
       <c r="P43" s="28" t="n">
         <f aca="false">O43</f>
-        <v>1839.3875</v>
+        <v>3284.1825</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
@@ -2364,7 +2399,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C45" s="16"/>
       <c r="D45" s="16"/>
@@ -2379,16 +2414,16 @@
       <c r="M45" s="16"/>
       <c r="N45" s="16"/>
       <c r="O45" s="16" t="n">
-        <v>719.1</v>
+        <v>559.3</v>
       </c>
       <c r="P45" s="22" t="n">
         <f aca="false">SUM(C45:O45)</f>
-        <v>719.1</v>
+        <v>559.3</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C46" s="24" t="n">
         <f aca="false">MAX(0,$B$12+C19-C45-C34)</f>
@@ -2424,19 +2459,19 @@
       </c>
       <c r="K46" s="24" t="n">
         <f aca="false">MAX(0,J46+K19-K45-K34)</f>
-        <v>479.4</v>
+        <v>639.2</v>
       </c>
       <c r="L46" s="24" t="n">
         <f aca="false">MAX(0,K46+L19-L45-L34)</f>
-        <v>799</v>
+        <v>639.2</v>
       </c>
       <c r="M46" s="24" t="n">
         <f aca="false">MAX(0,L46+M19-M45-M34)</f>
-        <v>719.1</v>
+        <v>559.3</v>
       </c>
       <c r="N46" s="24" t="n">
         <f aca="false">MAX(0,M46+N19-N45-N34)</f>
-        <v>719.1</v>
+        <v>559.3</v>
       </c>
       <c r="O46" s="24" t="n">
         <f aca="false">MAX(0,N46+O19-O45-O34)</f>
@@ -2445,92 +2480,92 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="D47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="E47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="F47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="G47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="H47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="I47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="J47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="K47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="L47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="M47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="N47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
       <c r="O47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>500</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="25" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C48" s="28" t="n">
         <f aca="false">C43-C46-C47</f>
-        <v>6000</v>
+        <v>4900</v>
       </c>
       <c r="D48" s="28" t="n">
         <f aca="false">D43-D46-D47</f>
-        <v>4850</v>
+        <v>3750</v>
       </c>
       <c r="E48" s="28" t="n">
         <f aca="false">E43-E46-E47</f>
-        <v>4200</v>
+        <v>3100</v>
       </c>
       <c r="F48" s="28" t="n">
         <f aca="false">F43-F46-F47</f>
-        <v>1200</v>
+        <v>100</v>
       </c>
       <c r="G48" s="28" t="n">
         <f aca="false">G43-G46-G47</f>
-        <v>800</v>
+        <v>-300</v>
       </c>
       <c r="H48" s="28" t="n">
         <f aca="false">H43-H46-H47</f>
-        <v>773</v>
+        <v>-327</v>
       </c>
       <c r="I48" s="28" t="n">
         <f aca="false">I43-I46-I47</f>
-        <v>849.8075</v>
+        <v>-250.1925</v>
       </c>
       <c r="J48" s="28" t="n">
         <f aca="false">J43-J46-J47</f>
@@ -2538,157 +2573,305 @@
       </c>
       <c r="K48" s="28" t="n">
         <f aca="false">K43-K46-K47</f>
-        <v>-482.09</v>
+        <v>-91.8900000000001</v>
       </c>
       <c r="L48" s="28" t="n">
         <f aca="false">L43-L46-L47</f>
-        <v>-317.555</v>
+        <v>647.45</v>
       </c>
       <c r="M48" s="28" t="n">
         <f aca="false">M43-M46-M47</f>
-        <v>-478.31</v>
+        <v>476.285</v>
       </c>
       <c r="N48" s="28" t="n">
         <f aca="false">N43-N46-N47</f>
-        <v>372.7825</v>
+        <v>477.3775</v>
       </c>
       <c r="O48" s="28" t="n">
         <f aca="false">O43-O46-O47</f>
-        <v>1339.3875</v>
+        <v>1684.1825</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="25" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C49" s="29" t="str">
-        <f aca="false">IF(C43&lt;0,"SOLDE NÉGATIF",IF(C43&lt;C47,"SOUS RÉSERVE MINI",IF(C48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
+        <f aca="false">IF($B$6="","à saisir",IF(C43&lt;0,"SOLDE NÉGATIF",IF(C43&lt;C47,"SOUS RÉSERVE MINI",IF(C48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
         <v>OK</v>
       </c>
       <c r="D49" s="29" t="str">
-        <f aca="false">IF(D43&lt;0,"SOLDE NÉGATIF",IF(D43&lt;D47,"SOUS RÉSERVE MINI",IF(D48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
+        <f aca="false">IF($B$6="","à saisir",IF(D43&lt;0,"SOLDE NÉGATIF",IF(D43&lt;D47,"SOUS RÉSERVE MINI",IF(D48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
         <v>OK</v>
       </c>
       <c r="E49" s="29" t="str">
-        <f aca="false">IF(E43&lt;0,"SOLDE NÉGATIF",IF(E43&lt;E47,"SOUS RÉSERVE MINI",IF(E48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
+        <f aca="false">IF($B$6="","à saisir",IF(E43&lt;0,"SOLDE NÉGATIF",IF(E43&lt;E47,"SOUS RÉSERVE MINI",IF(E48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
         <v>OK</v>
       </c>
       <c r="F49" s="29" t="str">
-        <f aca="false">IF(F43&lt;0,"SOLDE NÉGATIF",IF(F43&lt;F47,"SOUS RÉSERVE MINI",IF(F48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
+        <f aca="false">IF($B$6="","à saisir",IF(F43&lt;0,"SOLDE NÉGATIF",IF(F43&lt;F47,"SOUS RÉSERVE MINI",IF(F48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
         <v>OK</v>
       </c>
       <c r="G49" s="29" t="str">
-        <f aca="false">IF(G43&lt;0,"SOLDE NÉGATIF",IF(G43&lt;G47,"SOUS RÉSERVE MINI",IF(G48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
+        <f aca="false">IF($B$6="","à saisir",IF(G43&lt;0,"SOLDE NÉGATIF",IF(G43&lt;G47,"SOUS RÉSERVE MINI",IF(G48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>SOUS RÉSERVE MINI</v>
+      </c>
+      <c r="H49" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(H43&lt;0,"SOLDE NÉGATIF",IF(H43&lt;H47,"SOUS RÉSERVE MINI",IF(H48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>SOUS RÉSERVE MINI</v>
+      </c>
+      <c r="I49" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(I43&lt;0,"SOLDE NÉGATIF",IF(I43&lt;I47,"SOUS RÉSERVE MINI",IF(I48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>SOUS RÉSERVE MINI</v>
+      </c>
+      <c r="J49" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(J43&lt;0,"SOLDE NÉGATIF",IF(J43&lt;J47,"SOUS RÉSERVE MINI",IF(J48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
         <v>OK</v>
       </c>
-      <c r="H49" s="29" t="str">
-        <f aca="false">IF(H43&lt;0,"SOLDE NÉGATIF",IF(H43&lt;H47,"SOUS RÉSERVE MINI",IF(H48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
+      <c r="K49" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(K43&lt;0,"SOLDE NÉGATIF",IF(K43&lt;K47,"SOUS RÉSERVE MINI",IF(K48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>PRÉCOMMANDES NON COUVERTES</v>
+      </c>
+      <c r="L49" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(L43&lt;0,"SOLDE NÉGATIF",IF(L43&lt;L47,"SOUS RÉSERVE MINI",IF(L48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
         <v>OK</v>
       </c>
-      <c r="I49" s="29" t="str">
-        <f aca="false">IF(I43&lt;0,"SOLDE NÉGATIF",IF(I43&lt;I47,"SOUS RÉSERVE MINI",IF(I48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
+      <c r="M49" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(M43&lt;0,"SOLDE NÉGATIF",IF(M43&lt;M47,"SOUS RÉSERVE MINI",IF(M48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
         <v>OK</v>
       </c>
-      <c r="J49" s="29" t="str">
-        <f aca="false">IF(J43&lt;0,"SOLDE NÉGATIF",IF(J43&lt;J47,"SOUS RÉSERVE MINI",IF(J48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
+      <c r="N49" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(N43&lt;0,"SOLDE NÉGATIF",IF(N43&lt;N47,"SOUS RÉSERVE MINI",IF(N48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
         <v>OK</v>
       </c>
-      <c r="K49" s="29" t="str">
-        <f aca="false">IF(K43&lt;0,"SOLDE NÉGATIF",IF(K43&lt;K47,"SOUS RÉSERVE MINI",IF(K48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>SOUS RÉSERVE MINI</v>
-      </c>
-      <c r="L49" s="29" t="str">
-        <f aca="false">IF(L43&lt;0,"SOLDE NÉGATIF",IF(L43&lt;L47,"SOUS RÉSERVE MINI",IF(L48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>PRÉCOMMANDES NON COUVERTES</v>
-      </c>
-      <c r="M49" s="29" t="str">
-        <f aca="false">IF(M43&lt;0,"SOLDE NÉGATIF",IF(M43&lt;M47,"SOUS RÉSERVE MINI",IF(M48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>PRÉCOMMANDES NON COUVERTES</v>
-      </c>
-      <c r="N49" s="29" t="str">
-        <f aca="false">IF(N43&lt;0,"SOLDE NÉGATIF",IF(N43&lt;N47,"SOUS RÉSERVE MINI",IF(N48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
+      <c r="O49" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(O43&lt;0,"SOLDE NÉGATIF",IF(O43&lt;O47,"SOUS RÉSERVE MINI",IF(O48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
         <v>OK</v>
       </c>
-      <c r="O49" s="29" t="str">
-        <f aca="false">IF(O43&lt;0,"SOLDE NÉGATIF",IF(O43&lt;O47,"SOUS RÉSERVE MINI",IF(O48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF($B$6-$B$12&lt;$B$7,"OUI","non"))</f>
+        <v>non</v>
+      </c>
+      <c r="D50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(C48&lt;0,"OUI","non"))</f>
+        <v>non</v>
+      </c>
+      <c r="E50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(D48&lt;0,"OUI","non"))</f>
+        <v>non</v>
+      </c>
+      <c r="F50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(E48&lt;0,"OUI","non"))</f>
+        <v>non</v>
+      </c>
+      <c r="G50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(F48&lt;0,"OUI","non"))</f>
+        <v>non</v>
+      </c>
+      <c r="H50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(G48&lt;0,"OUI","non"))</f>
+        <v>OUI</v>
+      </c>
+      <c r="I50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(H48&lt;0,"OUI","non"))</f>
+        <v>OUI</v>
+      </c>
+      <c r="J50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(I48&lt;0,"OUI","non"))</f>
+        <v>OUI</v>
+      </c>
+      <c r="K50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(J48&lt;0,"OUI","non"))</f>
+        <v>non</v>
+      </c>
+      <c r="L50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(K48&lt;0,"OUI","non"))</f>
+        <v>OUI</v>
+      </c>
+      <c r="M50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(L48&lt;0,"OUI","non"))</f>
+        <v>non</v>
+      </c>
+      <c r="N50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(M48&lt;0,"OUI","non"))</f>
+        <v>non</v>
+      </c>
+      <c r="O50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(N48&lt;0,"OUI","non"))</f>
+        <v>non</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="B51" s="13"/>
-      <c r="C51" s="13"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="13"/>
-      <c r="G51" s="13"/>
-      <c r="H51" s="13"/>
-      <c r="I51" s="13"/>
-      <c r="J51" s="13"/>
-      <c r="K51" s="13"/>
-      <c r="L51" s="13"/>
-      <c r="M51" s="13"/>
-      <c r="N51" s="13"/>
-      <c r="O51" s="13"/>
-      <c r="P51" s="13"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="B52" s="27" t="n">
-        <f aca="false">MIN(C43:O43)</f>
-        <v>497.31</v>
+      <c r="A51" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51" s="22" t="n">
+        <f aca="false">IF(C50="OUI",C30+C35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="22" t="n">
+        <f aca="false">IF(D50="OUI",D30+D35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E51" s="22" t="n">
+        <f aca="false">IF(E50="OUI",E30+E35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="22" t="n">
+        <f aca="false">IF(F50="OUI",F30+F35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G51" s="22" t="n">
+        <f aca="false">IF(G50="OUI",G30+G35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H51" s="22" t="n">
+        <f aca="false">IF(H50="OUI",H30+H35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I51" s="22" t="n">
+        <f aca="false">IF(I50="OUI",I30+I35,0)</f>
+        <v>150</v>
+      </c>
+      <c r="J51" s="22" t="n">
+        <f aca="false">IF(J50="OUI",J30+J35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K51" s="22" t="n">
+        <f aca="false">IF(K50="OUI",K30+K35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L51" s="22" t="n">
+        <f aca="false">IF(L50="OUI",L30+L35,0)</f>
+        <v>150</v>
+      </c>
+      <c r="M51" s="22" t="n">
+        <f aca="false">IF(M50="OUI",M30+M35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N51" s="22" t="n">
+        <f aca="false">IF(N50="OUI",N30+N35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O51" s="22" t="n">
+        <f aca="false">IF(O50="OUI",O30+O35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P51" s="22" t="n">
+        <f aca="false">SUM(C51:O51)</f>
+        <v>300</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="B53" s="30" t="n">
-        <f aca="false">INDEX(C14:O14,MATCH(B52,C43:O43,0))</f>
-        <v>9</v>
-      </c>
+      <c r="A53" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B53" s="13"/>
+      <c r="C53" s="13"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="13"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="13"/>
+      <c r="I53" s="13"/>
+      <c r="J53" s="13"/>
+      <c r="K53" s="13"/>
+      <c r="L53" s="13"/>
+      <c r="M53" s="13"/>
+      <c r="N53" s="13"/>
+      <c r="O53" s="13"/>
+      <c r="P53" s="13"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="B54" s="30" t="n">
-        <f aca="false">COUNTIF(C49:O49,"&lt;&gt;OK")</f>
-        <v>3</v>
+        <v>90</v>
+      </c>
+      <c r="B54" s="27" t="n">
+        <f aca="false">MIN(C43:O43)</f>
+        <v>1273</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="B55" s="31" t="n">
+        <v>91</v>
+      </c>
+      <c r="B55" s="30" t="n">
+        <f aca="false">INDEX(C14:O14,MATCH(B54,C43:O43,0))</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B56" s="30" t="n">
+        <f aca="false">COUNTIF(C49:O49,"&lt;&gt;OK")-COUNTIF(C49:O49,"à saisir")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B57" s="31" t="n">
         <f aca="false">SUM(C22:O22)-SUM(C24:O24)</f>
         <v>1117.1625</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="B56" s="31" t="n">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="B58" s="31" t="n">
         <f aca="false">P21</f>
-        <v>191.65</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="B57" s="31" t="n">
+        <v>187.055</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="B59" s="31" t="n">
         <f aca="false">(P17+P19)*$B$11/(1+$B$11)</f>
-        <v>508.778908418131</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>91</v>
+        <v>496.804995374653</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="B60" s="30" t="n">
+        <f aca="false">COUNTIF(C50:O50,"OUI")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="B61" s="30" t="n">
+        <f aca="false">IF(B60=0,"aucune",INDEX(C14:O14,MATCH("OUI",C50:O50,0)))</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="B62" s="31" t="n">
+        <f aca="false">P51</f>
+        <v>300</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2696,13 +2879,23 @@
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="C49:O49">
-    <cfRule type="cellIs" priority="2" operator="notEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>"OK"</formula>
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND(C49&lt;&gt;"OK",C49&lt;&gt;"à saisir")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C50:O50">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"OUI"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C51:O51">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C43:O43">
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>C43&lt;C47</formula>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND($B$6&lt;&gt;"",C43&lt;C47)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -2726,7 +2919,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:P57"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -2737,17 +2930,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
@@ -2767,7 +2960,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -2787,89 +2980,91 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B6" s="16"/>
       <c r="C6" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="16"/>
+        <v>37</v>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>1600</v>
+      </c>
       <c r="C7" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>0.025</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>0.3</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B10" s="18" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B11" s="19" t="n">
         <v>0.081</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B12" s="16" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -2889,7 +3084,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B14" s="20"/>
       <c r="C14" s="20" t="n">
@@ -2932,12 +3127,12 @@
         <v>13</v>
       </c>
       <c r="P14" s="20" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C15" s="21" t="str">
         <f aca="false">IF($B$5="","",$B$5+7*(C$14-1))</f>
@@ -2994,7 +3189,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C16" s="21" t="str">
         <f aca="false">IF($B$5="","",C15+6)</f>
@@ -3051,7 +3246,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
@@ -3073,7 +3268,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="18"/>
@@ -3095,7 +3290,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
@@ -3117,7 +3312,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="18"/>
@@ -3139,7 +3334,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C21" s="24" t="n">
         <f aca="false">(C17+C19)*$B$8+(C18+C20)*$B$9</f>
@@ -3200,7 +3395,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C22" s="24" t="n">
         <f aca="false">C17+C19-C21</f>
@@ -3261,7 +3456,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
@@ -3281,7 +3476,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C24" s="24" t="n">
         <f aca="false">IF(C$14-$B$10&gt;=1,INDEX($C$22:$O$22,C$14-$B$10),0)</f>
@@ -3342,7 +3537,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
@@ -3364,7 +3559,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
@@ -3386,7 +3581,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="25" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C27" s="22" t="n">
         <f aca="false">C24+C25+C26</f>
@@ -3447,7 +3642,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
@@ -3467,7 +3662,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
@@ -3489,7 +3684,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
@@ -3511,7 +3706,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
@@ -3533,7 +3728,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
@@ -3555,7 +3750,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C33" s="16"/>
       <c r="D33" s="16"/>
@@ -3577,7 +3772,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C34" s="16"/>
       <c r="D34" s="16"/>
@@ -3599,7 +3794,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
@@ -3621,7 +3816,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
@@ -3643,7 +3838,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
@@ -3665,7 +3860,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>
@@ -3687,7 +3882,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="25" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C39" s="22" t="n">
         <f aca="false">SUM(C29:C38)</f>
@@ -3748,7 +3943,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
@@ -3768,7 +3963,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C41" s="24" t="n">
         <f aca="false">$B$6</f>
@@ -3829,7 +4024,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C42" s="26" t="n">
         <f aca="false">C27-C39</f>
@@ -3890,7 +4085,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="25" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C43" s="27" t="n">
         <f aca="false">C41+C42</f>
@@ -3951,7 +4146,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
@@ -3971,7 +4166,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C45" s="16"/>
       <c r="D45" s="16"/>
@@ -3993,7 +4188,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C46" s="24" t="n">
         <f aca="false">MAX(0,$B$12+C19-C45-C34)</f>
@@ -4050,250 +4245,398 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="D47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="E47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="F47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="G47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="H47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="I47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="J47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="K47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="L47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="M47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="N47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="O47" s="24" t="n">
         <f aca="false">$B$7</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="25" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C48" s="28" t="n">
         <f aca="false">C43-C46-C47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="D48" s="28" t="n">
         <f aca="false">D43-D46-D47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="E48" s="28" t="n">
         <f aca="false">E43-E46-E47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="F48" s="28" t="n">
         <f aca="false">F43-F46-F47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="G48" s="28" t="n">
         <f aca="false">G43-G46-G47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="H48" s="28" t="n">
         <f aca="false">H43-H46-H47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="I48" s="28" t="n">
         <f aca="false">I43-I46-I47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="J48" s="28" t="n">
         <f aca="false">J43-J46-J47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="K48" s="28" t="n">
         <f aca="false">K43-K46-K47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="L48" s="28" t="n">
         <f aca="false">L43-L46-L47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="M48" s="28" t="n">
         <f aca="false">M43-M46-M47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="N48" s="28" t="n">
         <f aca="false">N43-N46-N47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="O48" s="28" t="n">
         <f aca="false">O43-O46-O47</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="25" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C49" s="29" t="str">
-        <f aca="false">IF(C43&lt;0,"SOLDE NÉGATIF",IF(C43&lt;C47,"SOUS RÉSERVE MINI",IF(C48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(C43&lt;0,"SOLDE NÉGATIF",IF(C43&lt;C47,"SOUS RÉSERVE MINI",IF(C48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="D49" s="29" t="str">
-        <f aca="false">IF(D43&lt;0,"SOLDE NÉGATIF",IF(D43&lt;D47,"SOUS RÉSERVE MINI",IF(D48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(D43&lt;0,"SOLDE NÉGATIF",IF(D43&lt;D47,"SOUS RÉSERVE MINI",IF(D48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="E49" s="29" t="str">
-        <f aca="false">IF(E43&lt;0,"SOLDE NÉGATIF",IF(E43&lt;E47,"SOUS RÉSERVE MINI",IF(E48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(E43&lt;0,"SOLDE NÉGATIF",IF(E43&lt;E47,"SOUS RÉSERVE MINI",IF(E48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="F49" s="29" t="str">
-        <f aca="false">IF(F43&lt;0,"SOLDE NÉGATIF",IF(F43&lt;F47,"SOUS RÉSERVE MINI",IF(F48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(F43&lt;0,"SOLDE NÉGATIF",IF(F43&lt;F47,"SOUS RÉSERVE MINI",IF(F48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="G49" s="29" t="str">
-        <f aca="false">IF(G43&lt;0,"SOLDE NÉGATIF",IF(G43&lt;G47,"SOUS RÉSERVE MINI",IF(G48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(G43&lt;0,"SOLDE NÉGATIF",IF(G43&lt;G47,"SOUS RÉSERVE MINI",IF(G48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="H49" s="29" t="str">
-        <f aca="false">IF(H43&lt;0,"SOLDE NÉGATIF",IF(H43&lt;H47,"SOUS RÉSERVE MINI",IF(H48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(H43&lt;0,"SOLDE NÉGATIF",IF(H43&lt;H47,"SOUS RÉSERVE MINI",IF(H48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="I49" s="29" t="str">
-        <f aca="false">IF(I43&lt;0,"SOLDE NÉGATIF",IF(I43&lt;I47,"SOUS RÉSERVE MINI",IF(I48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(I43&lt;0,"SOLDE NÉGATIF",IF(I43&lt;I47,"SOUS RÉSERVE MINI",IF(I48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="J49" s="29" t="str">
-        <f aca="false">IF(J43&lt;0,"SOLDE NÉGATIF",IF(J43&lt;J47,"SOUS RÉSERVE MINI",IF(J48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(J43&lt;0,"SOLDE NÉGATIF",IF(J43&lt;J47,"SOUS RÉSERVE MINI",IF(J48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="K49" s="29" t="str">
-        <f aca="false">IF(K43&lt;0,"SOLDE NÉGATIF",IF(K43&lt;K47,"SOUS RÉSERVE MINI",IF(K48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(K43&lt;0,"SOLDE NÉGATIF",IF(K43&lt;K47,"SOUS RÉSERVE MINI",IF(K48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="L49" s="29" t="str">
-        <f aca="false">IF(L43&lt;0,"SOLDE NÉGATIF",IF(L43&lt;L47,"SOUS RÉSERVE MINI",IF(L48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(L43&lt;0,"SOLDE NÉGATIF",IF(L43&lt;L47,"SOUS RÉSERVE MINI",IF(L48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="M49" s="29" t="str">
-        <f aca="false">IF(M43&lt;0,"SOLDE NÉGATIF",IF(M43&lt;M47,"SOUS RÉSERVE MINI",IF(M48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(M43&lt;0,"SOLDE NÉGATIF",IF(M43&lt;M47,"SOUS RÉSERVE MINI",IF(M48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="N49" s="29" t="str">
-        <f aca="false">IF(N43&lt;0,"SOLDE NÉGATIF",IF(N43&lt;N47,"SOUS RÉSERVE MINI",IF(N48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(N43&lt;0,"SOLDE NÉGATIF",IF(N43&lt;N47,"SOUS RÉSERVE MINI",IF(N48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
       </c>
       <c r="O49" s="29" t="str">
-        <f aca="false">IF(O43&lt;0,"SOLDE NÉGATIF",IF(O43&lt;O47,"SOUS RÉSERVE MINI",IF(O48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK")))</f>
-        <v>OK</v>
+        <f aca="false">IF($B$6="","à saisir",IF(O43&lt;0,"SOLDE NÉGATIF",IF(O43&lt;O47,"SOUS RÉSERVE MINI",IF(O48&lt;0,"PRÉCOMMANDES NON COUVERTES","OK"))))</f>
+        <v>à saisir</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF($B$6-$B$12&lt;$B$7,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="D50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(C48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="E50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(D48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="F50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(E48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="G50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(F48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="H50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(G48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="I50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(H48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="J50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(I48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="K50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(J48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="L50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(K48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="M50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(L48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="N50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(M48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
+      </c>
+      <c r="O50" s="29" t="str">
+        <f aca="false">IF($B$6="","à saisir",IF(N48&lt;0,"OUI","non"))</f>
+        <v>à saisir</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="B51" s="13"/>
-      <c r="C51" s="13"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="13"/>
-      <c r="G51" s="13"/>
-      <c r="H51" s="13"/>
-      <c r="I51" s="13"/>
-      <c r="J51" s="13"/>
-      <c r="K51" s="13"/>
-      <c r="L51" s="13"/>
-      <c r="M51" s="13"/>
-      <c r="N51" s="13"/>
-      <c r="O51" s="13"/>
-      <c r="P51" s="13"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="B52" s="27" t="n">
-        <f aca="false">MIN(C43:O43)</f>
+      <c r="A51" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51" s="22" t="n">
+        <f aca="false">IF(C50="OUI",C30+C35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="22" t="n">
+        <f aca="false">IF(D50="OUI",D30+D35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E51" s="22" t="n">
+        <f aca="false">IF(E50="OUI",E30+E35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="22" t="n">
+        <f aca="false">IF(F50="OUI",F30+F35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G51" s="22" t="n">
+        <f aca="false">IF(G50="OUI",G30+G35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H51" s="22" t="n">
+        <f aca="false">IF(H50="OUI",H30+H35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I51" s="22" t="n">
+        <f aca="false">IF(I50="OUI",I30+I35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J51" s="22" t="n">
+        <f aca="false">IF(J50="OUI",J30+J35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K51" s="22" t="n">
+        <f aca="false">IF(K50="OUI",K30+K35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L51" s="22" t="n">
+        <f aca="false">IF(L50="OUI",L30+L35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M51" s="22" t="n">
+        <f aca="false">IF(M50="OUI",M30+M35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N51" s="22" t="n">
+        <f aca="false">IF(N50="OUI",N30+N35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O51" s="22" t="n">
+        <f aca="false">IF(O50="OUI",O30+O35,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P51" s="22" t="n">
+        <f aca="false">SUM(C51:O51)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="B53" s="30" t="n">
-        <f aca="false">INDEX(C14:O14,MATCH(B52,C43:O43,0))</f>
-        <v>1</v>
-      </c>
+      <c r="A53" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B53" s="13"/>
+      <c r="C53" s="13"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="13"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="13"/>
+      <c r="I53" s="13"/>
+      <c r="J53" s="13"/>
+      <c r="K53" s="13"/>
+      <c r="L53" s="13"/>
+      <c r="M53" s="13"/>
+      <c r="N53" s="13"/>
+      <c r="O53" s="13"/>
+      <c r="P53" s="13"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="B54" s="30" t="n">
-        <f aca="false">COUNTIF(C49:O49,"&lt;&gt;OK")</f>
+        <v>90</v>
+      </c>
+      <c r="B54" s="27" t="n">
+        <f aca="false">MIN(C43:O43)</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="B55" s="31" t="n">
-        <f aca="false">SUM(C22:O22)-SUM(C24:O24)</f>
-        <v>0</v>
+        <v>91</v>
+      </c>
+      <c r="B55" s="30" t="n">
+        <f aca="false">INDEX(C14:O14,MATCH(B54,C43:O43,0))</f>
+        <v>1</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="B56" s="31" t="n">
-        <f aca="false">P21</f>
+        <v>92</v>
+      </c>
+      <c r="B56" s="30" t="n">
+        <f aca="false">COUNTIF(C49:O49,"&lt;&gt;OK")-COUNTIF(C49:O49,"à saisir")</f>
         <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="25" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B57" s="31" t="n">
+        <f aca="false">SUM(C22:O22)-SUM(C24:O24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="B58" s="31" t="n">
+        <f aca="false">P21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="B59" s="31" t="n">
         <f aca="false">(P17+P19)*$B$11/(1+$B$11)</f>
         <v>0</v>
       </c>
-      <c r="C57" s="2" t="s">
-        <v>91</v>
+      <c r="C59" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="B60" s="30" t="n">
+        <f aca="false">COUNTIF(C50:O50,"OUI")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="B61" s="30" t="str">
+        <f aca="false">IF(B60=0,"aucune",INDEX(C14:O14,MATCH("OUI",C50:O50,0)))</f>
+        <v>aucune</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="B62" s="31" t="n">
+        <f aca="false">P51</f>
+        <v>0</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -4301,13 +4644,23 @@
     <mergeCell ref="A3:P3"/>
   </mergeCells>
   <conditionalFormatting sqref="C49:O49">
-    <cfRule type="cellIs" priority="2" operator="notEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>"OK"</formula>
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND(C49&lt;&gt;"OK",C49&lt;&gt;"à saisir")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C50:O50">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"OUI"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C51:O51">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C43:O43">
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>C43&lt;C47</formula>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND($B$6&lt;&gt;"",C43&lt;C47)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>